<commit_message>
Mantenedor de productos y desarrollo.
</commit_message>
<xml_diff>
--- a/public/database/Productos.xlsx
+++ b/public/database/Productos.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Productos" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:M1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,128 +410,39 @@
         <v>Descripcion</v>
       </c>
       <c r="D1" t="str">
+        <v>Categoria</v>
+      </c>
+      <c r="E1" t="str">
         <v>Valor</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>ValorOriginal</v>
+      </c>
+      <c r="G1" t="str">
         <v>Stock</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
+        <v>Activo</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Destacado</v>
+      </c>
+      <c r="J1" t="str">
+        <v>ConDescuento</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Orden</v>
+      </c>
+      <c r="L1" t="str">
         <v>ImageUrl</v>
       </c>
-      <c r="G1" t="str">
-        <v>ConDescuento</v>
-      </c>
-      <c r="H1" t="str">
+      <c r="M1" t="str">
         <v>VideoUrl</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>4</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Pijama 4</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Diseñados en colombia, piel de durazno.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>5</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2" t="str">
-        <v>https://rosmiyasc.s3.us-east-2.amazonaws.com/productos/000004/main.jpg</v>
-      </c>
-      <c r="G2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H2" t="str">
-        <v>/Producto1.mp4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Pijama 1</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Diseñados en colombia, piel de durazno.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3" t="str">
-        <v>https://rosmiyasc.s3.us-east-2.amazonaws.com/productos/000001/main.jpg</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="str">
-        <v>/Producto1.mp4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>19</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Pijama 19</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Diseñados en colombia, piel de durazno.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>7</v>
-      </c>
-      <c r="E4">
-        <v>10</v>
-      </c>
-      <c r="F4" t="str">
-        <v>productos/producto-1.webp</v>
-      </c>
-      <c r="G4" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4" t="str">
-        <v>/productos/producto-1.mp4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>9</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Pijama 9</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Diseñados en colombia, piel de durazno.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>10</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
-        <v>producto9.webp</v>
-      </c>
-      <c r="G5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" t="str">
-        <v>/Producto1.mp4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>